<commit_message>
Make overall Exia progress series visible
</commit_message>
<xml_diff>
--- a/Reports/Exia/build_progress_tracker_v1/exia_build_progress_tracker.xlsx
+++ b/Reports/Exia/build_progress_tracker_v1/exia_build_progress_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R55176f003ea14a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="2" r:id="R864d2c11e64e4a8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R41c2210299844e83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="4" r:id="R8c99621f6d1a4b58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R62d7e37f14b745bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="2" r:id="Ra95315debea54871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R07faf9bf3c4542d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="4" r:id="Ref67a12b57604f7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -309,45 +309,17 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Overall</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="111827"/>
-            </a:solidFill>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Chart Data'!$A$2:$A$9</c:f>
-              <c:strCache>
-                <c:ptCount val="0"/>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Chart Data'!$B$2:$B$9</c:f>
-              <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
             <c:v>Trend Up</c:v>
           </c:tx>
           <c:spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="16A34A"/>
             </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="16A34A"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -372,8 +344,8 @@
           <c:smooth val="0"/>
         </c:ser>
         <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:idx val="1"/>
+          <c:order val="1"/>
           <c:tx>
             <c:v>Trend Down</c:v>
           </c:tx>
@@ -381,6 +353,11 @@
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="DC2626"/>
             </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="DC2626"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -405,8 +382,8 @@
           <c:smooth val="0"/>
         </c:ser>
         <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
+          <c:idx val="2"/>
+          <c:order val="2"/>
           <c:tx>
             <c:v>Range / Neutral</c:v>
           </c:tx>
@@ -414,6 +391,11 @@
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="D97706"/>
             </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="D97706"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -429,6 +411,51 @@
           <c:val>
             <c:numRef>
               <c:f>'Chart Data'!$E$2:$E$9</c:f>
+              <c:numCache>
+                <c:formatCode>0.0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>Overall (all regimes)</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2563EB"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="38100">
+              <a:solidFill>
+                <a:srgbClr val="2563EB"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Data'!$A$2:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Data'!$B$2:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="0"/>
@@ -563,7 +590,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R85a3bd200be947ef"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re93ecc1203234ad5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -859,7 +886,7 @@
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="31" t="str">
-        <x:v>Метрика: средний stress-costed результат, bps на сделку/наблюдение. Более высокий mean не означает прохождение gate.</x:v>
+        <x:v>Метрика: средний stress-costed результат, bps на сделку/наблюдение. Синий пунктир Overall = результат по всем режимам; более высокий mean не означает прохождение gate.</x:v>
       </x:c>
       <x:c r="B3" s="31"/>
       <x:c r="C3" s="31"/>
@@ -1277,7 +1304,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R419a8e7379c449c3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b3c8432b11d4b09"/>
 </x:worksheet>
 </file>
 
@@ -1839,7 +1866,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9bc69cd1862479b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a0a9255edb84a0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2043,7 +2070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcd1d97b0b2f45af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2866a9c981d45e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>